<commit_message>
Update Step 4 Excel
</commit_message>
<xml_diff>
--- a/Article_data/Step 4 - Figure 2 data - Hotspot products.xlsx
+++ b/Article_data/Step 4 - Figure 2 data - Hotspot products.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\nicolas\projects\202604-paper-1-supplementary-code\Article_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E502AB90-5262-4035-B7EF-391E72D0C3C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{065C342E-700A-421D-9D77-47281D28365C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-30" windowWidth="29040" windowHeight="15720" xr2:uid="{3AE344CB-1894-47AD-A205-3A52A8D8A89E}"/>
+    <workbookView xWindow="-28920" yWindow="-30" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{3AE344CB-1894-47AD-A205-3A52A8D8A89E}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="2" r:id="rId1"/>

</xml_diff>